<commit_message>
feat: update institutional documents and add IP, OP, and major clinical procedures pages
</commit_message>
<xml_diff>
--- a/assets/xl/faculty-attendance.xlsx
+++ b/assets/xl/faculty-attendance.xlsx
@@ -270,7 +270,7 @@
               <color rgb="FF000000"/>
               <rFont val="Arial"/>
             </rPr>
-            <t xml:space="preserve">3/2/2026 2:21:08 PM</t>
+            <t xml:space="preserve">7/7/2026 9:47:54 AM</t>
           </r>
           <r>
             <rPr>
@@ -294,7 +294,7 @@
               <color rgb="FF000000"/>
               <rFont val="Arial"/>
             </rPr>
-            <t xml:space="preserve">DCI Admin</t>
+            <t xml:space="preserve">Malabar_nodal</t>
           </r>
         </is>
       </c>
@@ -470,28 +470,28 @@
       </c>
       <c s="6" t="inlineStr" r="G6">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H6">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I6">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J6">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c s="4" r="K6">
         <v>1</v>
       </c>
       <c s="6" t="inlineStr" r="L6">
         <is>
-          <t xml:space="preserve">150:53</t>
+          <t xml:space="preserve">167:58</t>
         </is>
       </c>
       <c s="7" r="M6">
-        <v>0.958333333333333</v>
+        <v>0.961538461538462</v>
       </c>
     </row>
     <row r="7" ht="17.9" customHeight="0">
@@ -505,48 +505,48 @@
       </c>
       <c s="5" t="inlineStr" r="C7">
         <is>
-          <t xml:space="preserve">Anusree G Nambiar</t>
+          <t xml:space="preserve">Gopika P Madhavan</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D7">
         <is>
-          <t xml:space="preserve">111100056799</t>
+          <t xml:space="preserve">111100038766</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E7">
         <is>
-          <t xml:space="preserve">Lecturer</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F7">
         <is>
-          <t xml:space="preserve">General Medicine</t>
+          <t xml:space="preserve">Prosthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G7">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H7">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I7">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J7">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c s="4" r="K7">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c s="6" t="inlineStr" r="L7">
         <is>
-          <t xml:space="preserve">147:50</t>
+          <t xml:space="preserve">165:59</t>
         </is>
       </c>
       <c s="7" r="M7">
-        <v>0.916666666666667</v>
+        <v>0.961538461538462</v>
       </c>
     </row>
     <row r="8" ht="17.85" customHeight="0">
@@ -560,12 +560,12 @@
       </c>
       <c s="5" t="inlineStr" r="C8">
         <is>
-          <t xml:space="preserve">Gayathri M J</t>
+          <t xml:space="preserve">Krishna Priya N</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D8">
         <is>
-          <t xml:space="preserve">111100038024</t>
+          <t xml:space="preserve">111100023144</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E8">
@@ -575,33 +575,33 @@
       </c>
       <c s="5" t="inlineStr" r="F8">
         <is>
-          <t xml:space="preserve">Orthodontics</t>
+          <t xml:space="preserve">Conservative Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G8">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H8">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I8">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J8">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c s="4" r="K8">
         <v>1</v>
       </c>
       <c s="6" t="inlineStr" r="L8">
         <is>
-          <t xml:space="preserve">146:58</t>
+          <t xml:space="preserve">160:14</t>
         </is>
       </c>
       <c s="7" r="M8">
-        <v>0.958333333333333</v>
+        <v>0.961538461538462</v>
       </c>
     </row>
     <row r="9" ht="17.9" customHeight="0">
@@ -615,48 +615,48 @@
       </c>
       <c s="5" t="inlineStr" r="C9">
         <is>
-          <t xml:space="preserve">Krishna Priya N</t>
+          <t xml:space="preserve">Beena M S</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D9">
         <is>
-          <t xml:space="preserve">111100023144</t>
+          <t xml:space="preserve">111100022391</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E9">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Assistant Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F9">
         <is>
-          <t xml:space="preserve">Conservative Dentistry</t>
+          <t xml:space="preserve">Pedodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G9">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H9">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I9">
+        <v>26</v>
+      </c>
+      <c s="4" r="J9">
         <v>24</v>
       </c>
-      <c s="4" r="J9">
-        <v>21</v>
-      </c>
       <c s="4" r="K9">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c s="6" t="inlineStr" r="L9">
         <is>
-          <t xml:space="preserve">144:24</t>
+          <t xml:space="preserve">160:03</t>
         </is>
       </c>
       <c s="7" r="M9">
-        <v>0.875</v>
+        <v>0.923076923076923</v>
       </c>
     </row>
     <row r="10" ht="17.85" customHeight="0">
@@ -670,12 +670,12 @@
       </c>
       <c s="5" t="inlineStr" r="C10">
         <is>
-          <t xml:space="preserve">Jiji V Unni</t>
+          <t xml:space="preserve">Greeshma Sudhakaran</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D10">
         <is>
-          <t xml:space="preserve">111100062384</t>
+          <t xml:space="preserve">111100038104</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E10">
@@ -685,33 +685,33 @@
       </c>
       <c s="5" t="inlineStr" r="F10">
         <is>
-          <t xml:space="preserve">Oral Medicine</t>
+          <t xml:space="preserve">Periodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G10">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H10">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I10">
+        <v>26</v>
+      </c>
+      <c s="4" r="J10">
         <v>24</v>
-      </c>
-      <c s="4" r="J10">
-        <v>22</v>
       </c>
       <c s="4" r="K10">
         <v>2</v>
       </c>
       <c s="6" t="inlineStr" r="L10">
         <is>
-          <t xml:space="preserve">138:02</t>
+          <t xml:space="preserve">159:37</t>
         </is>
       </c>
       <c s="7" r="M10">
-        <v>0.916666666666667</v>
+        <v>0.923076923076923</v>
       </c>
     </row>
     <row r="11" ht="17.9" customHeight="0">
@@ -725,48 +725,48 @@
       </c>
       <c s="5" t="inlineStr" r="C11">
         <is>
-          <t xml:space="preserve">Jishnu S</t>
+          <t xml:space="preserve">Abdul Vahab C P</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D11">
         <is>
-          <t xml:space="preserve">111100028717</t>
+          <t xml:space="preserve">111100022972</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E11">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F11">
         <is>
-          <t xml:space="preserve">Orthodontics</t>
+          <t xml:space="preserve">Microbiology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G11">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I11">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J11">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c s="4" r="K11">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c s="6" t="inlineStr" r="L11">
         <is>
-          <t xml:space="preserve">136:35</t>
+          <t xml:space="preserve">156:58</t>
         </is>
       </c>
       <c s="7" r="M11">
-        <v>0.833333333333333</v>
+        <v>0.961538461538462</v>
       </c>
     </row>
     <row r="12" ht="17.9" customHeight="0">
@@ -780,12 +780,12 @@
       </c>
       <c s="5" t="inlineStr" r="C12">
         <is>
-          <t xml:space="preserve">Shamna .C</t>
+          <t xml:space="preserve">Gayathri M J</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D12">
         <is>
-          <t xml:space="preserve">111100062395</t>
+          <t xml:space="preserve">111100038024</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E12">
@@ -795,33 +795,33 @@
       </c>
       <c s="5" t="inlineStr" r="F12">
         <is>
-          <t xml:space="preserve">Physiology</t>
+          <t xml:space="preserve">Orthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G12">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H12">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I12">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J12">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c s="4" r="K12">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c s="6" t="inlineStr" r="L12">
         <is>
-          <t xml:space="preserve">135:15</t>
+          <t xml:space="preserve">153:18</t>
         </is>
       </c>
       <c s="7" r="M12">
-        <v>0.875</v>
+        <v>0.961538461538462</v>
       </c>
     </row>
     <row r="13" ht="17.85" customHeight="0">
@@ -835,48 +835,48 @@
       </c>
       <c s="5" t="inlineStr" r="C13">
         <is>
-          <t xml:space="preserve">Ramya T R</t>
+          <t xml:space="preserve">Raihan Hariz</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D13">
         <is>
-          <t xml:space="preserve">111100066584</t>
+          <t xml:space="preserve">111100056774</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E13">
         <is>
-          <t xml:space="preserve">Lecturer</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F13">
         <is>
-          <t xml:space="preserve">Biochemistry</t>
+          <t xml:space="preserve">Oral Pathology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G13">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H13">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I13">
+        <v>26</v>
+      </c>
+      <c s="4" r="J13">
         <v>24</v>
-      </c>
-      <c s="4" r="J13">
-        <v>22</v>
       </c>
       <c s="4" r="K13">
         <v>2</v>
       </c>
       <c s="6" t="inlineStr" r="L13">
         <is>
-          <t xml:space="preserve">133:35</t>
+          <t xml:space="preserve">152:11</t>
         </is>
       </c>
       <c s="7" r="M13">
-        <v>0.916666666666667</v>
+        <v>0.923076923076923</v>
       </c>
     </row>
     <row r="14" ht="17.9" customHeight="0">
@@ -890,12 +890,12 @@
       </c>
       <c s="5" t="inlineStr" r="C14">
         <is>
-          <t xml:space="preserve">Greeshma Sudhakaran</t>
+          <t xml:space="preserve">Shahana Amjad Ali</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D14">
         <is>
-          <t xml:space="preserve">111100038104</t>
+          <t xml:space="preserve">111100043247</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E14">
@@ -905,33 +905,33 @@
       </c>
       <c s="5" t="inlineStr" r="F14">
         <is>
-          <t xml:space="preserve">Periodontics</t>
+          <t xml:space="preserve">Oral Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G14">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H14">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I14">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J14">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c s="4" r="K14">
         <v>3</v>
       </c>
       <c s="6" t="inlineStr" r="L14">
         <is>
-          <t xml:space="preserve">133:33</t>
+          <t xml:space="preserve">150:55</t>
         </is>
       </c>
       <c s="7" r="M14">
-        <v>0.875</v>
+        <v>0.884615384615385</v>
       </c>
     </row>
     <row r="15" ht="17.85" customHeight="0">
@@ -965,28 +965,28 @@
       </c>
       <c s="6" t="inlineStr" r="G15">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H15">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I15">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J15">
-        <v>20</v>
+        <v>25</v>
       </c>
       <c s="4" r="K15">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c s="6" t="inlineStr" r="L15">
         <is>
-          <t xml:space="preserve">132:00</t>
+          <t xml:space="preserve">147:53</t>
         </is>
       </c>
       <c s="7" r="M15">
-        <v>0.833333333333333</v>
+        <v>0.961538461538462</v>
       </c>
     </row>
     <row r="16" ht="17.9" customHeight="0">
@@ -1000,48 +1000,48 @@
       </c>
       <c s="5" t="inlineStr" r="C16">
         <is>
-          <t xml:space="preserve">Maneesha S J</t>
+          <t xml:space="preserve">Divya Mary Mathew</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D16">
         <is>
-          <t xml:space="preserve">111100038097</t>
+          <t xml:space="preserve">111100056796</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E16">
         <is>
-          <t xml:space="preserve">Lecturer</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F16">
         <is>
-          <t xml:space="preserve">Microbiology</t>
+          <t xml:space="preserve">Pedodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G16">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H16">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I16">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J16">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c s="4" r="K16">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c s="6" t="inlineStr" r="L16">
         <is>
-          <t xml:space="preserve">128:19</t>
+          <t xml:space="preserve">144:18</t>
         </is>
       </c>
       <c s="7" r="M16">
-        <v>0.875</v>
+        <v>0.846153846153846</v>
       </c>
     </row>
     <row r="17" ht="17.9" customHeight="0">
@@ -1055,12 +1055,12 @@
       </c>
       <c s="5" t="inlineStr" r="C17">
         <is>
-          <t xml:space="preserve">Amjad Ali</t>
+          <t xml:space="preserve">Jiji V Unni</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D17">
         <is>
-          <t xml:space="preserve">111100043245</t>
+          <t xml:space="preserve">111100062384</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E17">
@@ -1070,33 +1070,33 @@
       </c>
       <c s="5" t="inlineStr" r="F17">
         <is>
-          <t xml:space="preserve">Oral Surgery</t>
+          <t xml:space="preserve">Oral Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G17">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H17">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I17">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J17">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c s="4" r="K17">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c s="6" t="inlineStr" r="L17">
         <is>
-          <t xml:space="preserve">122:33</t>
+          <t xml:space="preserve">143:47</t>
         </is>
       </c>
       <c s="7" r="M17">
-        <v>0.791666666666667</v>
+        <v>0.846153846153846</v>
       </c>
     </row>
     <row r="18" ht="17.85" customHeight="0">
@@ -1110,12 +1110,12 @@
       </c>
       <c s="5" t="inlineStr" r="C18">
         <is>
-          <t xml:space="preserve">Divya Mary Mathew</t>
+          <t xml:space="preserve">Amjad Ali</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D18">
         <is>
-          <t xml:space="preserve">111100056796</t>
+          <t xml:space="preserve">111100043245</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E18">
@@ -1125,33 +1125,33 @@
       </c>
       <c s="5" t="inlineStr" r="F18">
         <is>
-          <t xml:space="preserve">Pedodontics</t>
+          <t xml:space="preserve">Oral Surgery</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G18">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H18">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I18">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J18">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c s="4" r="K18">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c s="6" t="inlineStr" r="L18">
         <is>
-          <t xml:space="preserve">120:16</t>
+          <t xml:space="preserve">142:26</t>
         </is>
       </c>
       <c s="7" r="M18">
-        <v>0.833333333333333</v>
+        <v>0.884615384615385</v>
       </c>
     </row>
     <row r="19" ht="17.9" customHeight="0">
@@ -1165,48 +1165,48 @@
       </c>
       <c s="5" t="inlineStr" r="C19">
         <is>
-          <t xml:space="preserve">Abdul Vahab C P</t>
+          <t xml:space="preserve">Arun Mohan</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D19">
         <is>
-          <t xml:space="preserve">111100022972</t>
+          <t xml:space="preserve">111100029118</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E19">
         <is>
-          <t xml:space="preserve">Lecturer</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F19">
         <is>
-          <t xml:space="preserve">Microbiology</t>
+          <t xml:space="preserve">Oral Pathology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G19">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H19">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I19">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J19">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c s="4" r="K19">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c s="6" t="inlineStr" r="L19">
         <is>
-          <t xml:space="preserve">118:56</t>
+          <t xml:space="preserve">140:50</t>
         </is>
       </c>
       <c s="7" r="M19">
-        <v>0.791666666666667</v>
+        <v>0.846153846153846</v>
       </c>
     </row>
     <row r="20" ht="17.85" customHeight="0">
@@ -1220,12 +1220,12 @@
       </c>
       <c s="5" t="inlineStr" r="C20">
         <is>
-          <t xml:space="preserve">Gopika P Madhavan</t>
+          <t xml:space="preserve">S Nandakumar</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D20">
         <is>
-          <t xml:space="preserve">111100038766</t>
+          <t xml:space="preserve">111100046680</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E20">
@@ -1240,28 +1240,28 @@
       </c>
       <c s="6" t="inlineStr" r="G20">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H20">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I20">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J20">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c s="4" r="K20">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c s="6" t="inlineStr" r="L20">
         <is>
-          <t xml:space="preserve">118:52</t>
+          <t xml:space="preserve">137:12</t>
         </is>
       </c>
       <c s="7" r="M20">
-        <v>0.75</v>
+        <v>0.846153846153846</v>
       </c>
     </row>
     <row r="21" ht="17.9" customHeight="0">
@@ -1275,48 +1275,48 @@
       </c>
       <c s="5" t="inlineStr" r="C21">
         <is>
-          <t xml:space="preserve">Sini V</t>
+          <t xml:space="preserve">M S Balakrishna</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D21">
         <is>
-          <t xml:space="preserve">111100044002</t>
+          <t xml:space="preserve">111100022481</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E21">
         <is>
-          <t xml:space="preserve">Assistant Professor</t>
+          <t xml:space="preserve">Professor &amp; HOD</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F21">
         <is>
-          <t xml:space="preserve">Anatomy</t>
+          <t xml:space="preserve">Oral Surgery</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G21">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H21">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I21">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J21">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c s="4" r="K21">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c s="6" t="inlineStr" r="L21">
         <is>
-          <t xml:space="preserve">116:22</t>
+          <t xml:space="preserve">135:35</t>
         </is>
       </c>
       <c s="7" r="M21">
-        <v>0.875</v>
+        <v>0.730769230769231</v>
       </c>
     </row>
     <row r="22" ht="17.85" customHeight="0">
@@ -1330,12 +1330,12 @@
       </c>
       <c s="5" t="inlineStr" r="C22">
         <is>
-          <t xml:space="preserve">Nikitha Mohan V J</t>
+          <t xml:space="preserve">Jishnu S</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D22">
         <is>
-          <t xml:space="preserve">111100056818</t>
+          <t xml:space="preserve">111100028717</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E22">
@@ -1345,33 +1345,33 @@
       </c>
       <c s="5" t="inlineStr" r="F22">
         <is>
-          <t xml:space="preserve">Community Dentistry</t>
+          <t xml:space="preserve">Orthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G22">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H22">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I22">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J22">
         <v>21</v>
       </c>
       <c s="4" r="K22">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c s="6" t="inlineStr" r="L22">
         <is>
-          <t xml:space="preserve">116:03</t>
+          <t xml:space="preserve">132:14</t>
         </is>
       </c>
       <c s="7" r="M22">
-        <v>0.875</v>
+        <v>0.807692307692308</v>
       </c>
     </row>
     <row r="23" ht="17.9" customHeight="0">
@@ -1385,12 +1385,12 @@
       </c>
       <c s="5" t="inlineStr" r="C23">
         <is>
-          <t xml:space="preserve">Shahana Amjad Ali</t>
+          <t xml:space="preserve">VRINDA M P</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D23">
         <is>
-          <t xml:space="preserve">111100043247</t>
+          <t xml:space="preserve">111100066577</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E23">
@@ -1400,33 +1400,33 @@
       </c>
       <c s="5" t="inlineStr" r="F23">
         <is>
-          <t xml:space="preserve">Oral Medicine</t>
+          <t xml:space="preserve">Pedodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G23">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H23">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I23">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J23">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c s="4" r="K23">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c s="6" t="inlineStr" r="L23">
         <is>
-          <t xml:space="preserve">115:13</t>
+          <t xml:space="preserve">131:02</t>
         </is>
       </c>
       <c s="7" r="M23">
-        <v>0.791666666666667</v>
+        <v>0.884615384615385</v>
       </c>
     </row>
     <row r="24" ht="17.9" customHeight="0">
@@ -1440,17 +1440,17 @@
       </c>
       <c s="5" t="inlineStr" r="C24">
         <is>
-          <t xml:space="preserve">Neethu Vins</t>
+          <t xml:space="preserve">Shamna .C</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D24">
         <is>
-          <t xml:space="preserve">111100062403</t>
+          <t xml:space="preserve">111100062395</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E24">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F24">
@@ -1460,28 +1460,28 @@
       </c>
       <c s="6" t="inlineStr" r="G24">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H24">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I24">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J24">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c s="4" r="K24">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c s="6" t="inlineStr" r="L24">
         <is>
-          <t xml:space="preserve">112:17</t>
+          <t xml:space="preserve">120:38</t>
         </is>
       </c>
       <c s="7" r="M24">
-        <v>0.666666666666667</v>
+        <v>0.884615384615385</v>
       </c>
     </row>
     <row r="25" ht="17.85" customHeight="0">
@@ -1495,17 +1495,17 @@
       </c>
       <c s="5" t="inlineStr" r="C25">
         <is>
-          <t xml:space="preserve">Suraj U</t>
+          <t xml:space="preserve">Alen Pius</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D25">
         <is>
-          <t xml:space="preserve">111100023438</t>
+          <t xml:space="preserve">111100043284</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E25">
         <is>
-          <t xml:space="preserve">Assistant Professor</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F25">
@@ -1515,28 +1515,28 @@
       </c>
       <c s="6" t="inlineStr" r="G25">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H25">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I25">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J25">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c s="4" r="K25">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c s="6" t="inlineStr" r="L25">
         <is>
-          <t xml:space="preserve">112:17</t>
+          <t xml:space="preserve">119:21</t>
         </is>
       </c>
       <c s="7" r="M25">
-        <v>0.791666666666667</v>
+        <v>0.615384615384615</v>
       </c>
     </row>
     <row r="26" ht="17.9" customHeight="0">
@@ -1550,48 +1550,48 @@
       </c>
       <c s="5" t="inlineStr" r="C26">
         <is>
-          <t xml:space="preserve">Neeraja K</t>
+          <t xml:space="preserve">ABDUL SAHEER P</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D26">
         <is>
-          <t xml:space="preserve">111100056857</t>
+          <t xml:space="preserve">111100022776</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E26">
         <is>
-          <t xml:space="preserve">Lecturer</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F26">
         <is>
-          <t xml:space="preserve">Conservative Dentistry</t>
+          <t xml:space="preserve">Community Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G26">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H26">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I26">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J26">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c s="4" r="K26">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c s="6" t="inlineStr" r="L26">
         <is>
-          <t xml:space="preserve">109:30</t>
+          <t xml:space="preserve">119:15</t>
         </is>
       </c>
       <c s="7" r="M26">
-        <v>0.875</v>
+        <v>0.846153846153846</v>
       </c>
     </row>
     <row r="27" ht="17.85" customHeight="0">
@@ -1605,17 +1605,17 @@
       </c>
       <c s="5" t="inlineStr" r="C27">
         <is>
-          <t xml:space="preserve">Alen Pius</t>
+          <t xml:space="preserve">Suraj U</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D27">
         <is>
-          <t xml:space="preserve">111100043284</t>
+          <t xml:space="preserve">111100023438</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E27">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Assistant Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F27">
@@ -1625,28 +1625,28 @@
       </c>
       <c s="6" t="inlineStr" r="G27">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H27">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I27">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J27">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c s="4" r="K27">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c s="6" t="inlineStr" r="L27">
         <is>
-          <t xml:space="preserve">109:15</t>
+          <t xml:space="preserve">113:40</t>
         </is>
       </c>
       <c s="7" r="M27">
-        <v>0.666666666666667</v>
+        <v>0.730769230769231</v>
       </c>
     </row>
     <row r="28" ht="17.9" customHeight="0">
@@ -1660,48 +1660,48 @@
       </c>
       <c s="5" t="inlineStr" r="C28">
         <is>
-          <t xml:space="preserve">Beena M S</t>
+          <t xml:space="preserve">Justin Ninan</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D28">
         <is>
-          <t xml:space="preserve">111100022391</t>
+          <t xml:space="preserve">111100023737</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E28">
         <is>
-          <t xml:space="preserve">Assistant Professor</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F28">
         <is>
-          <t xml:space="preserve">Pedodontics</t>
+          <t xml:space="preserve">Prosthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G28">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H28">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I28">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J28">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c s="4" r="K28">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c s="6" t="inlineStr" r="L28">
         <is>
-          <t xml:space="preserve">95:55</t>
+          <t xml:space="preserve">110:39</t>
         </is>
       </c>
       <c s="7" r="M28">
-        <v>0.791666666666667</v>
+        <v>0.692307692307692</v>
       </c>
     </row>
     <row r="29" ht="17.9" customHeight="0">
@@ -1735,28 +1735,28 @@
       </c>
       <c s="6" t="inlineStr" r="G29">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H29">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I29">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J29">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c s="4" r="K29">
         <v>10</v>
       </c>
       <c s="6" t="inlineStr" r="L29">
         <is>
-          <t xml:space="preserve">94:44</t>
+          <t xml:space="preserve">107:06</t>
         </is>
       </c>
       <c s="7" r="M29">
-        <v>0.583333333333333</v>
+        <v>0.615384615384615</v>
       </c>
     </row>
     <row r="30" ht="17.85" customHeight="0">
@@ -1770,48 +1770,48 @@
       </c>
       <c s="5" t="inlineStr" r="C30">
         <is>
-          <t xml:space="preserve">Feba Maria Varghese</t>
+          <t xml:space="preserve">Naveen O P</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D30">
         <is>
-          <t xml:space="preserve">111100062394</t>
+          <t xml:space="preserve">111100056890</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E30">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F30">
         <is>
-          <t xml:space="preserve">Prosthodontics</t>
+          <t xml:space="preserve">Oral Surgery</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G30">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H30">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I30">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J30">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c s="4" r="K30">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c s="6" t="inlineStr" r="L30">
         <is>
-          <t xml:space="preserve">93:25</t>
+          <t xml:space="preserve">103:00</t>
         </is>
       </c>
       <c s="7" r="M30">
-        <v>0.625</v>
+        <v>0.692307692307692</v>
       </c>
     </row>
     <row r="31" ht="17.9" customHeight="0">
@@ -1825,48 +1825,48 @@
       </c>
       <c s="5" t="inlineStr" r="C31">
         <is>
-          <t xml:space="preserve">Ramna T R</t>
+          <t xml:space="preserve">Reshma Rajan</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D31">
         <is>
-          <t xml:space="preserve">111100062387</t>
+          <t xml:space="preserve">111100037361</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E31">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F31">
         <is>
-          <t xml:space="preserve">Oral Pathology</t>
+          <t xml:space="preserve">Pedodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G31">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H31">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I31">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J31">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c s="4" r="K31">
-        <v>2</v>
+        <v>10</v>
       </c>
       <c s="6" t="inlineStr" r="L31">
         <is>
-          <t xml:space="preserve">92:21</t>
+          <t xml:space="preserve">100:24</t>
         </is>
       </c>
       <c s="7" r="M31">
-        <v>0.916666666666667</v>
+        <v>0.615384615384615</v>
       </c>
     </row>
     <row r="32" ht="17.85" customHeight="0">
@@ -1880,48 +1880,48 @@
       </c>
       <c s="5" t="inlineStr" r="C32">
         <is>
-          <t xml:space="preserve">Sayi D. S.</t>
+          <t xml:space="preserve">Neeraja K</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D32">
         <is>
-          <t xml:space="preserve">111100043330</t>
+          <t xml:space="preserve">111100056857</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E32">
         <is>
-          <t xml:space="preserve">Professor &amp; HOD</t>
+          <t xml:space="preserve">Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F32">
         <is>
-          <t xml:space="preserve">Microbiology</t>
+          <t xml:space="preserve">Conservative Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G32">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H32">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I32">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J32">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c s="4" r="K32">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c s="6" t="inlineStr" r="L32">
         <is>
-          <t xml:space="preserve">90:45</t>
+          <t xml:space="preserve">87:38</t>
         </is>
       </c>
       <c s="7" r="M32">
-        <v>0.666666666666667</v>
+        <v>0.769230769230769</v>
       </c>
     </row>
     <row r="33" ht="17.9" customHeight="0">
@@ -1935,17 +1935,17 @@
       </c>
       <c s="5" t="inlineStr" r="C33">
         <is>
-          <t xml:space="preserve">Arun Mohan</t>
+          <t xml:space="preserve">Ramna T R</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D33">
         <is>
-          <t xml:space="preserve">111100029118</t>
+          <t xml:space="preserve">111100062387</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E33">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F33">
@@ -1955,28 +1955,28 @@
       </c>
       <c s="6" t="inlineStr" r="G33">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H33">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I33">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J33">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c s="4" r="K33">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c s="6" t="inlineStr" r="L33">
         <is>
-          <t xml:space="preserve">88:44</t>
+          <t xml:space="preserve">85:52</t>
         </is>
       </c>
       <c s="7" r="M33">
-        <v>0.75</v>
+        <v>0.884615384615385</v>
       </c>
     </row>
     <row r="34" ht="17.85" customHeight="0">
@@ -1990,48 +1990,48 @@
       </c>
       <c s="5" t="inlineStr" r="C34">
         <is>
-          <t xml:space="preserve">Raihan Hariz</t>
+          <t xml:space="preserve">CHITHRA P</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D34">
         <is>
-          <t xml:space="preserve">111100056774</t>
+          <t xml:space="preserve">111100038011</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E34">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F34">
         <is>
-          <t xml:space="preserve">Oral Pathology</t>
+          <t xml:space="preserve">Oral Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G34">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H34">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I34">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J34">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c s="4" r="K34">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c s="6" t="inlineStr" r="L34">
         <is>
-          <t xml:space="preserve">85:14</t>
+          <t xml:space="preserve">83:35</t>
         </is>
       </c>
       <c s="7" r="M34">
-        <v>0.833333333333333</v>
+        <v>0.730769230769231</v>
       </c>
     </row>
     <row r="35" ht="17.9" customHeight="0">
@@ -2045,48 +2045,48 @@
       </c>
       <c s="5" t="inlineStr" r="C35">
         <is>
-          <t xml:space="preserve">M S Balakrishna</t>
+          <t xml:space="preserve">AJISH.M.SAJI</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D35">
         <is>
-          <t xml:space="preserve">111100022481</t>
+          <t xml:space="preserve">111100022470</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E35">
         <is>
-          <t xml:space="preserve">Professor &amp; HOD</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F35">
         <is>
-          <t xml:space="preserve">Oral Surgery</t>
+          <t xml:space="preserve">Oral Pathology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G35">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H35">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I35">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J35">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c s="4" r="K35">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c s="6" t="inlineStr" r="L35">
         <is>
-          <t xml:space="preserve">85:02</t>
+          <t xml:space="preserve">77:40</t>
         </is>
       </c>
       <c s="7" r="M35">
-        <v>0.541666666666667</v>
+        <v>0.615384615384615</v>
       </c>
     </row>
     <row r="36" ht="17.9" customHeight="0">
@@ -2100,48 +2100,48 @@
       </c>
       <c s="5" t="inlineStr" r="C36">
         <is>
-          <t xml:space="preserve">Emil George</t>
+          <t xml:space="preserve">Sayi D. S.</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D36">
         <is>
-          <t xml:space="preserve">111100062388</t>
+          <t xml:space="preserve">111100043330</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E36">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Professor &amp; HOD</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F36">
         <is>
-          <t xml:space="preserve">Conservative Dentistry</t>
+          <t xml:space="preserve">Microbiology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G36">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H36">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I36">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J36">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c s="4" r="K36">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c s="6" t="inlineStr" r="L36">
         <is>
-          <t xml:space="preserve">84:55</t>
+          <t xml:space="preserve">76:22</t>
         </is>
       </c>
       <c s="7" r="M36">
-        <v>0.5</v>
+        <v>0.615384615384615</v>
       </c>
     </row>
     <row r="37" ht="17.85" customHeight="0">
@@ -2155,48 +2155,48 @@
       </c>
       <c s="5" t="inlineStr" r="C37">
         <is>
-          <t xml:space="preserve">Anjana Vipal</t>
+          <t xml:space="preserve">Parson Paul</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D37">
         <is>
-          <t xml:space="preserve">111100062393</t>
+          <t xml:space="preserve">111100038022</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E37">
         <is>
-          <t xml:space="preserve">Lecturer</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F37">
         <is>
-          <t xml:space="preserve">Community Dentistry</t>
+          <t xml:space="preserve">Orthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G37">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H37">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I37">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J37">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c s="4" r="K37">
         <v>9</v>
       </c>
       <c s="6" t="inlineStr" r="L37">
         <is>
-          <t xml:space="preserve">81:49</t>
+          <t xml:space="preserve">74:42</t>
         </is>
       </c>
       <c s="7" r="M37">
-        <v>0.625</v>
+        <v>0.653846153846154</v>
       </c>
     </row>
     <row r="38" ht="17.9" customHeight="0">
@@ -2210,48 +2210,48 @@
       </c>
       <c s="5" t="inlineStr" r="C38">
         <is>
-          <t xml:space="preserve">Nita Syam</t>
+          <t xml:space="preserve">Neethu Vins</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D38">
         <is>
-          <t xml:space="preserve">111100039118</t>
+          <t xml:space="preserve">111100062403</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E38">
         <is>
-          <t xml:space="preserve">Professor &amp; HOD</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F38">
         <is>
-          <t xml:space="preserve">Periodontics</t>
+          <t xml:space="preserve">Physiology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G38">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H38">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I38">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J38">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c s="4" r="K38">
         <v>11</v>
       </c>
       <c s="6" t="inlineStr" r="L38">
         <is>
-          <t xml:space="preserve">81:45</t>
+          <t xml:space="preserve">73:28</t>
         </is>
       </c>
       <c s="7" r="M38">
-        <v>0.541666666666667</v>
+        <v>0.576923076923077</v>
       </c>
     </row>
     <row r="39" ht="17.85" customHeight="0">
@@ -2265,48 +2265,48 @@
       </c>
       <c s="5" t="inlineStr" r="C39">
         <is>
-          <t xml:space="preserve">Naveen O P</t>
+          <t xml:space="preserve">Sonu Ravindran</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D39">
         <is>
-          <t xml:space="preserve">111100056890</t>
+          <t xml:space="preserve">111100023435</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E39">
         <is>
-          <t xml:space="preserve">Professor</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F39">
         <is>
-          <t xml:space="preserve">Oral Surgery</t>
+          <t xml:space="preserve">Conservative Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G39">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H39">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I39">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J39">
+        <v>12</v>
+      </c>
+      <c s="4" r="K39">
         <v>14</v>
       </c>
-      <c s="4" r="K39">
-        <v>10</v>
-      </c>
       <c s="6" t="inlineStr" r="L39">
         <is>
-          <t xml:space="preserve">81:05</t>
+          <t xml:space="preserve">72:50</t>
         </is>
       </c>
       <c s="7" r="M39">
-        <v>0.583333333333333</v>
+        <v>0.461538461538462</v>
       </c>
     </row>
     <row r="40" ht="17.9" customHeight="0">
@@ -2320,48 +2320,48 @@
       </c>
       <c s="5" t="inlineStr" r="C40">
         <is>
-          <t xml:space="preserve">Justin Ninan</t>
+          <t xml:space="preserve">Shabeer Ahamed</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D40">
         <is>
-          <t xml:space="preserve">111100023737</t>
+          <t xml:space="preserve">111100022890</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E40">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Professor &amp; HOD</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F40">
         <is>
-          <t xml:space="preserve">Prosthodontics</t>
+          <t xml:space="preserve">Periodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G40">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H40">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I40">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J40">
-        <v>18</v>
+        <v>12</v>
       </c>
       <c s="4" r="K40">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c s="6" t="inlineStr" r="L40">
         <is>
-          <t xml:space="preserve">76:54</t>
+          <t xml:space="preserve">69:42</t>
         </is>
       </c>
       <c s="7" r="M40">
-        <v>0.75</v>
+        <v>0.461538461538462</v>
       </c>
     </row>
     <row r="41" ht="17.85" customHeight="0">
@@ -2375,48 +2375,48 @@
       </c>
       <c s="5" t="inlineStr" r="C41">
         <is>
-          <t xml:space="preserve">Sujith K</t>
+          <t xml:space="preserve">Mohammed Yasin KK</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D41">
         <is>
-          <t xml:space="preserve">111100038004</t>
+          <t xml:space="preserve">111100014494</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E41">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F41">
         <is>
-          <t xml:space="preserve">Prosthodontics</t>
+          <t xml:space="preserve">Conservative Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G41">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H41">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I41">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J41">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c s="4" r="K41">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c s="6" t="inlineStr" r="L41">
         <is>
-          <t xml:space="preserve">74:04</t>
+          <t xml:space="preserve">69:01</t>
         </is>
       </c>
       <c s="7" r="M41">
-        <v>0.75</v>
+        <v>0.384615384615385</v>
       </c>
     </row>
     <row r="42" ht="17.9" customHeight="0">
@@ -2430,17 +2430,17 @@
       </c>
       <c s="5" t="inlineStr" r="C42">
         <is>
-          <t xml:space="preserve">Sonu Ravindran</t>
+          <t xml:space="preserve">Vivek S B</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D42">
         <is>
-          <t xml:space="preserve">111100023435</t>
+          <t xml:space="preserve">111100056854</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E42">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F42">
@@ -2450,28 +2450,28 @@
       </c>
       <c s="6" t="inlineStr" r="G42">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H42">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I42">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J42">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c s="4" r="K42">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c s="6" t="inlineStr" r="L42">
         <is>
-          <t xml:space="preserve">72:49</t>
+          <t xml:space="preserve">68:40</t>
         </is>
       </c>
       <c s="7" r="M42">
-        <v>0.5</v>
+        <v>0.692307692307692</v>
       </c>
     </row>
     <row r="43" ht="17.9" customHeight="0">
@@ -2485,48 +2485,48 @@
       </c>
       <c s="5" t="inlineStr" r="C43">
         <is>
-          <t xml:space="preserve">Mohammed Yasin KK</t>
+          <t xml:space="preserve">Sujith K</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D43">
         <is>
-          <t xml:space="preserve">111100014494</t>
+          <t xml:space="preserve">111100038004</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E43">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F43">
         <is>
-          <t xml:space="preserve">Conservative Dentistry</t>
+          <t xml:space="preserve">Prosthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G43">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H43">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I43">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J43">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c s="4" r="K43">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c s="6" t="inlineStr" r="L43">
         <is>
-          <t xml:space="preserve">70:26</t>
+          <t xml:space="preserve">62:06</t>
         </is>
       </c>
       <c s="7" r="M43">
-        <v>0.416666666666667</v>
+        <v>0.692307692307692</v>
       </c>
     </row>
     <row r="44" ht="17.85" customHeight="0">
@@ -2540,48 +2540,48 @@
       </c>
       <c s="5" t="inlineStr" r="C44">
         <is>
-          <t xml:space="preserve">ABDUL SAHEER P</t>
+          <t xml:space="preserve">Ramya T R</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D44">
         <is>
-          <t xml:space="preserve">111100022776</t>
+          <t xml:space="preserve">111100066584</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E44">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F44">
         <is>
-          <t xml:space="preserve">Community Dentistry</t>
+          <t xml:space="preserve">Biochemistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G44">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H44">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I44">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J44">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c s="4" r="K44">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c s="6" t="inlineStr" r="L44">
         <is>
-          <t xml:space="preserve">68:00</t>
+          <t xml:space="preserve">57:11</t>
         </is>
       </c>
       <c s="7" r="M44">
-        <v>0.666666666666667</v>
+        <v>0.807692307692308</v>
       </c>
     </row>
     <row r="45" ht="17.9" customHeight="0">
@@ -2595,48 +2595,48 @@
       </c>
       <c s="5" t="inlineStr" r="C45">
         <is>
-          <t xml:space="preserve">Rasool Karim Nizaro Siyo</t>
+          <t xml:space="preserve">Nikitha Mohan V J</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D45">
         <is>
-          <t xml:space="preserve">111100022586</t>
+          <t xml:space="preserve">111100056818</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E45">
         <is>
-          <t xml:space="preserve">Professor &amp; HOD</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F45">
         <is>
-          <t xml:space="preserve">Orthodontics</t>
+          <t xml:space="preserve">Community Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G45">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H45">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I45">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J45">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c s="4" r="K45">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c s="6" t="inlineStr" r="L45">
         <is>
-          <t xml:space="preserve">62:39</t>
+          <t xml:space="preserve">42:23</t>
         </is>
       </c>
       <c s="7" r="M45">
-        <v>0.416666666666667</v>
+        <v>0.269230769230769</v>
       </c>
     </row>
     <row r="46" ht="17.85" customHeight="0">
@@ -2650,48 +2650,48 @@
       </c>
       <c s="5" t="inlineStr" r="C46">
         <is>
-          <t xml:space="preserve">S Nandakumar</t>
+          <t xml:space="preserve">Jeethu John Jerry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D46">
         <is>
-          <t xml:space="preserve">111100046680</t>
+          <t xml:space="preserve">111100028287</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E46">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F46">
         <is>
-          <t xml:space="preserve">Prosthodontics</t>
+          <t xml:space="preserve">Periodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G46">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H46">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I46">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J46">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c s="4" r="K46">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c s="6" t="inlineStr" r="L46">
         <is>
-          <t xml:space="preserve">61:09</t>
+          <t xml:space="preserve">40:43</t>
         </is>
       </c>
       <c s="7" r="M46">
-        <v>0.416666666666667</v>
+        <v>0.346153846153846</v>
       </c>
     </row>
     <row r="47" ht="17.9" customHeight="0">
@@ -2705,48 +2705,48 @@
       </c>
       <c s="5" t="inlineStr" r="C47">
         <is>
-          <t xml:space="preserve">Jeethu John Jerry</t>
+          <t xml:space="preserve">Sini V</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D47">
         <is>
-          <t xml:space="preserve">111100028287</t>
+          <t xml:space="preserve">111100044002</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E47">
         <is>
-          <t xml:space="preserve">Professor</t>
+          <t xml:space="preserve">Assistant Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F47">
         <is>
-          <t xml:space="preserve">Periodontics</t>
+          <t xml:space="preserve">Anatomy</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G47">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H47">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I47">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J47">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c s="4" r="K47">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c s="6" t="inlineStr" r="L47">
         <is>
-          <t xml:space="preserve">51:43</t>
+          <t xml:space="preserve">38:42</t>
         </is>
       </c>
       <c s="7" r="M47">
-        <v>0.5</v>
+        <v>0.615384615384615</v>
       </c>
     </row>
     <row r="48" ht="17.9" customHeight="0">
@@ -2760,48 +2760,48 @@
       </c>
       <c s="5" t="inlineStr" r="C48">
         <is>
-          <t xml:space="preserve">Reshma Rajan</t>
+          <t xml:space="preserve">Emil George</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D48">
         <is>
-          <t xml:space="preserve">111100037361</t>
+          <t xml:space="preserve">111100062388</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E48">
         <is>
-          <t xml:space="preserve">Professor</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F48">
         <is>
-          <t xml:space="preserve">Pedodontics</t>
+          <t xml:space="preserve">Conservative Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G48">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H48">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I48">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J48">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c s="4" r="K48">
-        <v>13</v>
+        <v>22</v>
       </c>
       <c s="6" t="inlineStr" r="L48">
         <is>
-          <t xml:space="preserve">37:52</t>
+          <t xml:space="preserve">29:19</t>
         </is>
       </c>
       <c s="7" r="M48">
-        <v>0.458333333333333</v>
+        <v>0.153846153846154</v>
       </c>
     </row>
     <row r="49" ht="17.85" customHeight="0">
@@ -2835,28 +2835,28 @@
       </c>
       <c s="6" t="inlineStr" r="G49">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H49">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I49">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J49">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c s="4" r="K49">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c s="6" t="inlineStr" r="L49">
         <is>
-          <t xml:space="preserve">34:13</t>
+          <t xml:space="preserve">18:55</t>
         </is>
       </c>
       <c s="7" r="M49">
-        <v>0.458333333333333</v>
+        <v>0.230769230769231</v>
       </c>
     </row>
     <row r="50" ht="17.9" customHeight="0">
@@ -2870,48 +2870,48 @@
       </c>
       <c s="5" t="inlineStr" r="C50">
         <is>
-          <t xml:space="preserve">Shabeer Ahamed</t>
+          <t xml:space="preserve">Bejoy Pulayampatt Unni</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D50">
         <is>
-          <t xml:space="preserve">111100022890</t>
+          <t xml:space="preserve">111100066506</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E50">
         <is>
-          <t xml:space="preserve">Professor &amp; HOD</t>
+          <t xml:space="preserve">Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F50">
         <is>
-          <t xml:space="preserve">Periodontics</t>
+          <t xml:space="preserve">Orthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G50">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H50">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I50">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J50">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c s="4" r="K50">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c s="6" t="inlineStr" r="L50">
         <is>
-          <t xml:space="preserve">31:19</t>
+          <t xml:space="preserve">06:10</t>
         </is>
       </c>
       <c s="7" r="M50">
-        <v>0.291666666666667</v>
+        <v>0.153846153846154</v>
       </c>
     </row>
     <row r="51" ht="17.85" customHeight="0">
@@ -2925,48 +2925,48 @@
       </c>
       <c s="5" t="inlineStr" r="C51">
         <is>
-          <t xml:space="preserve">Parson Paul</t>
+          <t xml:space="preserve">Maneesha S J</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D51">
         <is>
-          <t xml:space="preserve">111100038022</t>
+          <t xml:space="preserve">111100038097</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E51">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F51">
         <is>
-          <t xml:space="preserve">Orthodontics</t>
+          <t xml:space="preserve">Microbiology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G51">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H51">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I51">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J51">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c s="4" r="K51">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c s="6" t="inlineStr" r="L51">
         <is>
-          <t xml:space="preserve">30:14</t>
+          <t xml:space="preserve">06:03</t>
         </is>
       </c>
       <c s="7" r="M51">
-        <v>0.541666666666667</v>
+        <v>0.769230769230769</v>
       </c>
     </row>
     <row r="52" ht="17.9" customHeight="0">
@@ -2980,48 +2980,48 @@
       </c>
       <c s="5" t="inlineStr" r="C52">
         <is>
-          <t xml:space="preserve">Fathimath Zahra</t>
+          <t xml:space="preserve">Abdul Sameeh</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D52">
         <is>
-          <t xml:space="preserve">111100022430</t>
+          <t xml:space="preserve">111100056867</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E52">
         <is>
-          <t xml:space="preserve">Assistant Professor</t>
+          <t xml:space="preserve">Reader</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F52">
         <is>
-          <t xml:space="preserve">Oral Medicine</t>
+          <t xml:space="preserve">Prosthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G52">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H52">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I52">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J52">
-        <v>16</v>
+        <v>0</v>
       </c>
       <c s="4" r="K52">
-        <v>8</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L52">
         <is>
-          <t xml:space="preserve">20:03</t>
+          <t xml:space="preserve">00:00</t>
         </is>
       </c>
       <c s="7" r="M52">
-        <v>0.666666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="53" ht="17.85" customHeight="0">
@@ -3035,17 +3035,17 @@
       </c>
       <c s="5" t="inlineStr" r="C53">
         <is>
-          <t xml:space="preserve">Bejoy Pulayampatt Unni</t>
+          <t xml:space="preserve">Anjali N</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D53">
         <is>
-          <t xml:space="preserve">111100066506</t>
+          <t xml:space="preserve">111100023571</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E53">
         <is>
-          <t xml:space="preserve">Professor</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F53">
@@ -3055,28 +3055,28 @@
       </c>
       <c s="6" t="inlineStr" r="G53">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H53">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I53">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J53">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c s="4" r="K53">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L53">
         <is>
-          <t xml:space="preserve">13:21</t>
+          <t xml:space="preserve">00:00</t>
         </is>
       </c>
       <c s="7" r="M53">
-        <v>0.166666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="54" ht="17.9" customHeight="0">
@@ -3090,48 +3090,48 @@
       </c>
       <c s="5" t="inlineStr" r="C54">
         <is>
-          <t xml:space="preserve">AJISH.M.SAJI</t>
+          <t xml:space="preserve">Anjana Vipal</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D54">
         <is>
-          <t xml:space="preserve">111100022470</t>
+          <t xml:space="preserve">111100062393</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E54">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F54">
         <is>
-          <t xml:space="preserve">Oral Pathology</t>
+          <t xml:space="preserve">Community Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G54">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H54">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I54">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J54">
-        <v>13</v>
+        <v>0</v>
       </c>
       <c s="4" r="K54">
-        <v>11</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L54">
         <is>
-          <t xml:space="preserve">12:01</t>
+          <t xml:space="preserve">00:00</t>
         </is>
       </c>
       <c s="7" r="M54">
-        <v>0.541666666666667</v>
+        <v>0</v>
       </c>
     </row>
     <row r="55" ht="17.9" customHeight="0">
@@ -3145,40 +3145,40 @@
       </c>
       <c s="5" t="inlineStr" r="C55">
         <is>
-          <t xml:space="preserve">Abdul Sameeh</t>
+          <t xml:space="preserve">Anusree G Nambiar</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D55">
         <is>
-          <t xml:space="preserve">111100056867</t>
+          <t xml:space="preserve">111100056799</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E55">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F55">
         <is>
-          <t xml:space="preserve">Prosthodontics</t>
+          <t xml:space="preserve">General Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G55">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H55">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I55">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J55">
         <v>0</v>
       </c>
       <c s="4" r="K55">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L55">
         <is>
@@ -3200,12 +3200,12 @@
       </c>
       <c s="5" t="inlineStr" r="C56">
         <is>
-          <t xml:space="preserve">Anjali N</t>
+          <t xml:space="preserve">Anusree Sadanandan</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D56">
         <is>
-          <t xml:space="preserve">111100023571</t>
+          <t xml:space="preserve">111100038101</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E56">
@@ -3215,25 +3215,25 @@
       </c>
       <c s="5" t="inlineStr" r="F56">
         <is>
-          <t xml:space="preserve">Orthodontics</t>
+          <t xml:space="preserve">Pedodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G56">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H56">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I56">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J56">
         <v>0</v>
       </c>
       <c s="4" r="K56">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L56">
         <is>
@@ -3255,40 +3255,40 @@
       </c>
       <c s="5" t="inlineStr" r="C57">
         <is>
-          <t xml:space="preserve">Anusree Sadanandan</t>
+          <t xml:space="preserve">Deepak Daryani</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D57">
         <is>
-          <t xml:space="preserve">111100038101</t>
+          <t xml:space="preserve">111100022446</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E57">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Professor &amp; HOD</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F57">
         <is>
-          <t xml:space="preserve">Pedodontics</t>
+          <t xml:space="preserve">Oral Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G57">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H57">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I57">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J57">
         <v>0</v>
       </c>
       <c s="4" r="K57">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L57">
         <is>
@@ -3310,12 +3310,12 @@
       </c>
       <c s="5" t="inlineStr" r="C58">
         <is>
-          <t xml:space="preserve">CHITHRA P</t>
+          <t xml:space="preserve">Denis Paul K</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D58">
         <is>
-          <t xml:space="preserve">111100038011</t>
+          <t xml:space="preserve">111100056766</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E58">
@@ -3325,25 +3325,25 @@
       </c>
       <c s="5" t="inlineStr" r="F58">
         <is>
-          <t xml:space="preserve">Oral Medicine</t>
+          <t xml:space="preserve">Pedodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G58">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H58">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I58">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J58">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c s="4" r="K58">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L58">
         <is>
@@ -3351,7 +3351,7 @@
         </is>
       </c>
       <c s="7" r="M58">
-        <v>0.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="59" ht="17.9" customHeight="0">
@@ -3365,12 +3365,12 @@
       </c>
       <c s="5" t="inlineStr" r="C59">
         <is>
-          <t xml:space="preserve">Deepak Daryani</t>
+          <t xml:space="preserve">Dr Sabir Muliyar</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D59">
         <is>
-          <t xml:space="preserve">111100022446</t>
+          <t xml:space="preserve">111100015944</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E59">
@@ -3380,25 +3380,25 @@
       </c>
       <c s="5" t="inlineStr" r="F59">
         <is>
-          <t xml:space="preserve">Oral Medicine</t>
+          <t xml:space="preserve">Conservative Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G59">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H59">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I59">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J59">
         <v>0</v>
       </c>
       <c s="4" r="K59">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c s="6" t="inlineStr" r="L59">
         <is>
@@ -3420,40 +3420,40 @@
       </c>
       <c s="5" t="inlineStr" r="C60">
         <is>
-          <t xml:space="preserve">Denis Paul K</t>
+          <t xml:space="preserve">Fathimath Zahra</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D60">
         <is>
-          <t xml:space="preserve">111100056766</t>
+          <t xml:space="preserve">111100022430</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E60">
         <is>
-          <t xml:space="preserve">Reader</t>
+          <t xml:space="preserve">Assistant Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F60">
         <is>
-          <t xml:space="preserve">Pedodontics</t>
+          <t xml:space="preserve">Oral Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G60">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H60">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I60">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J60">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c s="4" r="K60">
-        <v>24</v>
+        <v>7</v>
       </c>
       <c s="6" t="inlineStr" r="L60">
         <is>
@@ -3461,7 +3461,7 @@
         </is>
       </c>
       <c s="7" r="M60">
-        <v>0</v>
+        <v>0.730769230769231</v>
       </c>
     </row>
     <row r="61" ht="17.85" customHeight="0">
@@ -3495,20 +3495,20 @@
       </c>
       <c s="6" t="inlineStr" r="G61">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H61">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I61">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J61">
         <v>0</v>
       </c>
       <c s="4" r="K61">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L61">
         <is>
@@ -3530,12 +3530,12 @@
       </c>
       <c s="5" t="inlineStr" r="C62">
         <is>
-          <t xml:space="preserve">Fouziya Begum</t>
+          <t xml:space="preserve">Feba Maria Varghese</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D62">
         <is>
-          <t xml:space="preserve">111100056873</t>
+          <t xml:space="preserve">111100062394</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E62">
@@ -3550,20 +3550,20 @@
       </c>
       <c s="6" t="inlineStr" r="G62">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H62">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I62">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J62">
         <v>0</v>
       </c>
       <c s="4" r="K62">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L62">
         <is>
@@ -3585,40 +3585,40 @@
       </c>
       <c s="5" t="inlineStr" r="C63">
         <is>
-          <t xml:space="preserve">Geetha Muniswamy</t>
+          <t xml:space="preserve">Fouziya Begum</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D63">
         <is>
-          <t xml:space="preserve">111100022454</t>
+          <t xml:space="preserve">111100056873</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E63">
         <is>
-          <t xml:space="preserve">Professor</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F63">
         <is>
-          <t xml:space="preserve">Pharmacology</t>
+          <t xml:space="preserve">Prosthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G63">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H63">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I63">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J63">
         <v>0</v>
       </c>
       <c s="4" r="K63">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L63">
         <is>
@@ -3640,12 +3640,12 @@
       </c>
       <c s="5" t="inlineStr" r="C64">
         <is>
-          <t xml:space="preserve">Gopinath K V</t>
+          <t xml:space="preserve">Geetha Muniswamy</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D64">
         <is>
-          <t xml:space="preserve">111100023297</t>
+          <t xml:space="preserve">111100022454</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E64">
@@ -3655,25 +3655,25 @@
       </c>
       <c s="5" t="inlineStr" r="F64">
         <is>
-          <t xml:space="preserve">General Surgery</t>
+          <t xml:space="preserve">Pharmacology</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G64">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H64">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I64">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J64">
         <v>0</v>
       </c>
       <c s="4" r="K64">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L64">
         <is>
@@ -3695,40 +3695,40 @@
       </c>
       <c s="5" t="inlineStr" r="C65">
         <is>
-          <t xml:space="preserve">Habeebulla Hassan</t>
+          <t xml:space="preserve">Gopinath K V</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D65">
         <is>
-          <t xml:space="preserve">111100056887</t>
+          <t xml:space="preserve">111100023297</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E65">
         <is>
-          <t xml:space="preserve">Tutor</t>
+          <t xml:space="preserve">Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F65">
         <is>
-          <t xml:space="preserve">General Medicine</t>
+          <t xml:space="preserve">General Surgery</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G65">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H65">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I65">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J65">
         <v>0</v>
       </c>
       <c s="4" r="K65">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L65">
         <is>
@@ -3750,12 +3750,12 @@
       </c>
       <c s="5" t="inlineStr" r="C66">
         <is>
-          <t xml:space="preserve">Helna Sidheeque</t>
+          <t xml:space="preserve">Habeebulla Hassan</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D66">
         <is>
-          <t xml:space="preserve">111100062390</t>
+          <t xml:space="preserve">111100056887</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E66">
@@ -3765,25 +3765,25 @@
       </c>
       <c s="5" t="inlineStr" r="F66">
         <is>
-          <t xml:space="preserve">Community Dentistry</t>
+          <t xml:space="preserve">General Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G66">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H66">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I66">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J66">
         <v>0</v>
       </c>
       <c s="4" r="K66">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L66">
         <is>
@@ -3805,40 +3805,40 @@
       </c>
       <c s="5" t="inlineStr" r="C67">
         <is>
-          <t xml:space="preserve">Ligil A R</t>
+          <t xml:space="preserve">Helna Sidheeque</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D67">
         <is>
-          <t xml:space="preserve">111100056823</t>
+          <t xml:space="preserve">111100062390</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E67">
         <is>
-          <t xml:space="preserve">Professor</t>
+          <t xml:space="preserve">Tutor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F67">
         <is>
-          <t xml:space="preserve">Orthodontics</t>
+          <t xml:space="preserve">Community Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G67">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H67">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I67">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J67">
         <v>0</v>
       </c>
       <c s="4" r="K67">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L67">
         <is>
@@ -3860,40 +3860,40 @@
       </c>
       <c s="5" t="inlineStr" r="C68">
         <is>
-          <t xml:space="preserve">Mariya Hashimi C K</t>
+          <t xml:space="preserve">Ligil A R</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D68">
         <is>
-          <t xml:space="preserve">111100043948</t>
+          <t xml:space="preserve">111100056823</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E68">
         <is>
-          <t xml:space="preserve">Lecturer</t>
+          <t xml:space="preserve">Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F68">
         <is>
-          <t xml:space="preserve">Biochemistry</t>
+          <t xml:space="preserve">Orthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G68">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H68">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I68">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J68">
         <v>0</v>
       </c>
       <c s="4" r="K68">
-        <v>20</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L68">
         <is>
@@ -3915,12 +3915,12 @@
       </c>
       <c s="5" t="inlineStr" r="C69">
         <is>
-          <t xml:space="preserve">Muhsina E</t>
+          <t xml:space="preserve">MEGHA J NAIR</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D69">
         <is>
-          <t xml:space="preserve">111100056897</t>
+          <t xml:space="preserve">111100010610</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E69">
@@ -3930,25 +3930,25 @@
       </c>
       <c s="5" t="inlineStr" r="F69">
         <is>
-          <t xml:space="preserve">Orthodontics</t>
+          <t xml:space="preserve">Periodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G69">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H69">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I69">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J69">
         <v>0</v>
       </c>
       <c s="4" r="K69">
-        <v>24</v>
+        <v>11</v>
       </c>
       <c s="6" t="inlineStr" r="L69">
         <is>
@@ -3970,12 +3970,12 @@
       </c>
       <c s="5" t="inlineStr" r="C70">
         <is>
-          <t xml:space="preserve">Nazreen P V</t>
+          <t xml:space="preserve">Muhsina E</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D70">
         <is>
-          <t xml:space="preserve">111100062385</t>
+          <t xml:space="preserve">111100056897</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E70">
@@ -3985,25 +3985,25 @@
       </c>
       <c s="5" t="inlineStr" r="F70">
         <is>
-          <t xml:space="preserve">Prosthodontics</t>
+          <t xml:space="preserve">Orthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G70">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H70">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I70">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J70">
         <v>0</v>
       </c>
       <c s="4" r="K70">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L70">
         <is>
@@ -4025,12 +4025,12 @@
       </c>
       <c s="5" t="inlineStr" r="C71">
         <is>
-          <t xml:space="preserve">Pooja Pramod Shetye</t>
+          <t xml:space="preserve">Nazreen P V</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D71">
         <is>
-          <t xml:space="preserve">111100062389</t>
+          <t xml:space="preserve">111100062385</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E71">
@@ -4040,25 +4040,25 @@
       </c>
       <c s="5" t="inlineStr" r="F71">
         <is>
-          <t xml:space="preserve">Conservative Dentistry</t>
+          <t xml:space="preserve">Prosthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G71">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H71">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I71">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J71">
         <v>0</v>
       </c>
       <c s="4" r="K71">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L71">
         <is>
@@ -4080,40 +4080,40 @@
       </c>
       <c s="5" t="inlineStr" r="C72">
         <is>
-          <t xml:space="preserve">Pradeep Kumar C</t>
+          <t xml:space="preserve">Pooja Pramod Shetye</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D72">
         <is>
-          <t xml:space="preserve">111100062386</t>
+          <t xml:space="preserve">111100062389</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E72">
         <is>
-          <t xml:space="preserve">Principal</t>
+          <t xml:space="preserve">Sr. Lecturer</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F72">
         <is>
-          <t xml:space="preserve">Prosthodontics</t>
+          <t xml:space="preserve">Conservative Dentistry</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G72">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H72">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I72">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J72">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c s="4" r="K72">
-        <v>9</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L72">
         <is>
@@ -4121,7 +4121,7 @@
         </is>
       </c>
       <c s="7" r="M72">
-        <v>0.625</v>
+        <v>0</v>
       </c>
     </row>
     <row r="73" ht="17.9" customHeight="0">
@@ -4135,17 +4135,17 @@
       </c>
       <c s="5" t="inlineStr" r="C73">
         <is>
-          <t xml:space="preserve">Punya Krishnan B</t>
+          <t xml:space="preserve">Pradeep Kumar C</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D73">
         <is>
-          <t xml:space="preserve">111100022792</t>
+          <t xml:space="preserve">111100062386</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E73">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Principal</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F73">
@@ -4155,20 +4155,20 @@
       </c>
       <c s="6" t="inlineStr" r="G73">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H73">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I73">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J73">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c s="4" r="K73">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c s="6" t="inlineStr" r="L73">
         <is>
@@ -4176,7 +4176,7 @@
         </is>
       </c>
       <c s="7" r="M73">
-        <v>0</v>
+        <v>0.307692307692308</v>
       </c>
     </row>
     <row r="74" ht="17.9" customHeight="0">
@@ -4210,20 +4210,20 @@
       </c>
       <c s="6" t="inlineStr" r="G74">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H74">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I74">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J74">
         <v>0</v>
       </c>
       <c s="4" r="K74">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L74">
         <is>
@@ -4245,40 +4245,40 @@
       </c>
       <c s="5" t="inlineStr" r="C75">
         <is>
-          <t xml:space="preserve">Sachin Venugopal Menon</t>
+          <t xml:space="preserve">Rasool Karim Nizaro Siyo</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D75">
         <is>
-          <t xml:space="preserve">111100023664</t>
+          <t xml:space="preserve">111100022586</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E75">
         <is>
-          <t xml:space="preserve">Professor</t>
+          <t xml:space="preserve">Professor &amp; HOD</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F75">
         <is>
-          <t xml:space="preserve">Genral Medicine</t>
+          <t xml:space="preserve">Orthodontics</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G75">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H75">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I75">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J75">
         <v>0</v>
       </c>
       <c s="4" r="K75">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L75">
         <is>
@@ -4300,40 +4300,40 @@
       </c>
       <c s="5" t="inlineStr" r="C76">
         <is>
-          <t xml:space="preserve">Sandhya Krishna M</t>
+          <t xml:space="preserve">Sachin Venugopal Menon</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="D76">
         <is>
-          <t xml:space="preserve">111100028302</t>
+          <t xml:space="preserve">111100023664</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="E76">
         <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
+          <t xml:space="preserve">Professor</t>
         </is>
       </c>
       <c s="5" t="inlineStr" r="F76">
         <is>
-          <t xml:space="preserve">Oral Medicine</t>
+          <t xml:space="preserve">Genral Medicine</t>
         </is>
       </c>
       <c s="6" t="inlineStr" r="G76">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H76">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I76">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J76">
         <v>0</v>
       </c>
       <c s="4" r="K76">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L76">
         <is>
@@ -4375,20 +4375,20 @@
       </c>
       <c s="6" t="inlineStr" r="G77">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H77">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I77">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J77">
         <v>0</v>
       </c>
       <c s="4" r="K77">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L77">
         <is>
@@ -4399,7 +4399,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="78" ht="17.9" customHeight="0">
+    <row r="78" ht="17.85" customHeight="0">
       <c s="4" r="A78">
         <v>73</v>
       </c>
@@ -4430,20 +4430,20 @@
       </c>
       <c s="6" t="inlineStr" r="G78">
         <is>
-          <t xml:space="preserve">02/2026</t>
+          <t xml:space="preserve">06/2026</t>
         </is>
       </c>
       <c s="4" r="H78">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c s="4" r="I78">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="4" r="J78">
         <v>0</v>
       </c>
       <c s="4" r="K78">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c s="6" t="inlineStr" r="L78">
         <is>
@@ -4454,116 +4454,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="79" ht="17.9" customHeight="0">
-      <c s="4" r="A79">
-        <v>74</v>
-      </c>
-      <c s="5" t="inlineStr" r="B79">
-        <is>
-          <t xml:space="preserve">Malabar Dental College And Research Centre, Malappuram</t>
-        </is>
-      </c>
-      <c s="5" t="inlineStr" r="C79">
-        <is>
-          <t xml:space="preserve">Vivek S B</t>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D79">
-        <is>
-          <t xml:space="preserve">111100056854</t>
-        </is>
-      </c>
-      <c s="5" t="inlineStr" r="E79">
-        <is>
-          <t xml:space="preserve">Lecturer</t>
-        </is>
-      </c>
-      <c s="5" t="inlineStr" r="F79">
-        <is>
-          <t xml:space="preserve">Conservative Dentistry</t>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="G79">
-        <is>
-          <t xml:space="preserve">02/2026</t>
-        </is>
-      </c>
-      <c s="4" r="H79">
-        <v>28</v>
-      </c>
-      <c s="4" r="I79">
-        <v>24</v>
-      </c>
-      <c s="4" r="J79">
-        <v>0</v>
-      </c>
-      <c s="4" r="K79">
-        <v>24</v>
-      </c>
-      <c s="6" t="inlineStr" r="L79">
-        <is>
-          <t xml:space="preserve">00:00</t>
-        </is>
-      </c>
-      <c s="7" r="M79">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" ht="17.85" customHeight="0">
-      <c s="4" r="A80">
-        <v>75</v>
-      </c>
-      <c s="5" t="inlineStr" r="B80">
-        <is>
-          <t xml:space="preserve">Malabar Dental College And Research Centre, Malappuram</t>
-        </is>
-      </c>
-      <c s="5" t="inlineStr" r="C80">
-        <is>
-          <t xml:space="preserve">VRINDA M P</t>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="D80">
-        <is>
-          <t xml:space="preserve">111100066577</t>
-        </is>
-      </c>
-      <c s="5" t="inlineStr" r="E80">
-        <is>
-          <t xml:space="preserve">Sr. Lecturer</t>
-        </is>
-      </c>
-      <c s="5" t="inlineStr" r="F80">
-        <is>
-          <t xml:space="preserve">Pedodontics</t>
-        </is>
-      </c>
-      <c s="6" t="inlineStr" r="G80">
-        <is>
-          <t xml:space="preserve">02/2026</t>
-        </is>
-      </c>
-      <c s="4" r="H80">
-        <v>28</v>
-      </c>
-      <c s="4" r="I80">
-        <v>24</v>
-      </c>
-      <c s="4" r="J80">
-        <v>0</v>
-      </c>
-      <c s="4" r="K80">
-        <v>24</v>
-      </c>
-      <c s="6" t="inlineStr" r="L80">
-        <is>
-          <t xml:space="preserve">00:00</t>
-        </is>
-      </c>
-      <c s="7" r="M80">
-        <v>0</v>
-      </c>
-    </row>
+    <row r="79" ht="0.05" customHeight="1"/>
   </sheetData>
   <mergeCells>
     <mergeCell ref="A1:M1"/>

</xml_diff>